<commit_message>
This is changes from Yesterday
</commit_message>
<xml_diff>
--- a/SAS_TD_FileAudit.xlsx
+++ b/SAS_TD_FileAudit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BDC\Projects\SASZombieAssaultTD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E1B0667-BA38-4EC3-8D66-6B89E748DF9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30049327-7D68-46D3-AE3B-DEBC61A9EF42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C829CA00-B181-41AF-960D-2C8D57D250F8}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="195">
   <si>
     <t>FileName</t>
   </si>
@@ -554,9 +554,6 @@
   </si>
   <si>
     <t>Engine/Systems/Assets</t>
-  </si>
-  <si>
-    <t>New File</t>
   </si>
   <si>
     <t>Strongly-typed asset identifier</t>
@@ -1570,7 +1567,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>20</v>
@@ -1582,7 +1579,7 @@
         <v>19</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F3" s="5"/>
     </row>
@@ -2167,193 +2164,213 @@
         <v>1</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>38</v>
+        <v>175</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>39</v>
+        <v>176</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F36" s="5"/>
+      <c r="F36" s="5" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="b">
         <v>1</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>41</v>
+        <v>178</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>42</v>
+        <v>176</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F37" s="5"/>
+      <c r="F37" s="5" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="b">
         <v>1</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>43</v>
+        <v>180</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>44</v>
+        <v>176</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F38" s="5"/>
+      <c r="F38" s="5" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="b">
         <v>1</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>45</v>
+        <v>182</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>46</v>
+        <v>176</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F39" s="5"/>
+      <c r="F39" s="5" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="b">
         <v>1</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>48</v>
+        <v>184</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>49</v>
+        <v>176</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F40" s="5"/>
+      <c r="F40" s="5" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="b">
         <v>1</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>51</v>
+        <v>186</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>52</v>
+        <v>176</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F41" s="5"/>
+      <c r="F41" s="5" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="b">
         <v>1</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>53</v>
+        <v>188</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>54</v>
+        <v>176</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F42" s="5"/>
+      <c r="F42" s="5" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="b">
         <v>1</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>55</v>
+        <v>190</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>56</v>
+        <v>176</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F43" s="5"/>
+      <c r="F43" s="5" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="b">
         <v>1</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>57</v>
+        <v>192</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>58</v>
+        <v>176</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F44" s="5"/>
+      <c r="F44" s="5" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="b">
         <v>1</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>61</v>
+        <v>176</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F45" s="5"/>
+      <c r="F45" s="5" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="b">
         <v>1</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>12</v>
@@ -2365,13 +2382,13 @@
         <v>1</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>12</v>
@@ -2383,13 +2400,13 @@
         <v>1</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>69</v>
+        <v>43</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>70</v>
+        <v>44</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>12</v>
@@ -2401,13 +2418,13 @@
         <v>1</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>71</v>
+        <v>45</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>12</v>
@@ -2419,13 +2436,13 @@
         <v>1</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>12</v>
@@ -2437,13 +2454,13 @@
         <v>1</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>12</v>
@@ -2455,13 +2472,13 @@
         <v>1</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>77</v>
+        <v>53</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>12</v>
@@ -2473,13 +2490,13 @@
         <v>1</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>12</v>
@@ -2491,13 +2508,13 @@
         <v>1</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>82</v>
+        <v>57</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>83</v>
+        <v>58</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>12</v>
@@ -2509,13 +2526,13 @@
         <v>1</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>84</v>
+        <v>60</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>12</v>
@@ -2527,13 +2544,13 @@
         <v>1</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>89</v>
+        <v>62</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>90</v>
+        <v>63</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>91</v>
+        <v>59</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>12</v>
@@ -2545,13 +2562,13 @@
         <v>1</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>93</v>
+        <v>65</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>94</v>
+        <v>59</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>12</v>
@@ -2563,13 +2580,13 @@
         <v>1</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>12</v>
@@ -2581,13 +2598,13 @@
         <v>1</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>97</v>
+        <v>71</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>12</v>
@@ -2599,13 +2616,13 @@
         <v>1</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>12</v>
@@ -2617,13 +2634,13 @@
         <v>1</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>106</v>
+        <v>76</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>12</v>
@@ -2635,13 +2652,13 @@
         <v>1</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>113</v>
+        <v>78</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>111</v>
+        <v>79</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>12</v>
@@ -2653,13 +2670,13 @@
         <v>1</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>121</v>
+        <v>81</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>111</v>
+        <v>79</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>12</v>
@@ -2671,13 +2688,13 @@
         <v>1</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>122</v>
+        <v>82</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>123</v>
+        <v>83</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>124</v>
+        <v>79</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>12</v>
@@ -2689,13 +2706,13 @@
         <v>1</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>125</v>
+        <v>84</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>126</v>
+        <v>85</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>124</v>
+        <v>79</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>12</v>
@@ -2707,13 +2724,13 @@
         <v>1</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>129</v>
+        <v>89</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>130</v>
+        <v>90</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>124</v>
+        <v>91</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>12</v>
@@ -2725,13 +2742,13 @@
         <v>1</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>131</v>
+        <v>92</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>132</v>
+        <v>93</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>12</v>
@@ -2743,13 +2760,13 @@
         <v>1</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>133</v>
+        <v>95</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>134</v>
+        <v>96</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>12</v>
@@ -2761,13 +2778,13 @@
         <v>1</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>135</v>
+        <v>97</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>136</v>
+        <v>98</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>12</v>
@@ -2779,13 +2796,13 @@
         <v>1</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>140</v>
+        <v>99</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>142</v>
+        <v>94</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>12</v>
@@ -2797,13 +2814,13 @@
         <v>1</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>143</v>
+        <v>105</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>144</v>
+        <v>106</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>142</v>
+        <v>94</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>12</v>
@@ -2815,13 +2832,13 @@
         <v>1</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>145</v>
+        <v>112</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>146</v>
+        <v>113</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>142</v>
+        <v>111</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>12</v>
@@ -2833,13 +2850,13 @@
         <v>1</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>148</v>
+        <v>121</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>142</v>
+        <v>111</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>12</v>
@@ -2851,13 +2868,13 @@
         <v>1</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>158</v>
+        <v>122</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>159</v>
+        <v>123</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>151</v>
+        <v>124</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>12</v>
@@ -2869,13 +2886,13 @@
         <v>1</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>171</v>
+        <v>125</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>164</v>
+        <v>124</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>12</v>
@@ -2887,206 +2904,190 @@
         <v>1</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>175</v>
+        <v>129</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>176</v>
+        <v>130</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>19</v>
+        <v>124</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F76" s="5" t="s">
-        <v>178</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F76" s="5"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="b">
         <v>1</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>179</v>
+        <v>131</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>176</v>
+        <v>132</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>19</v>
+        <v>124</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F77" s="5" t="s">
-        <v>180</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F77" s="5"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="b">
         <v>1</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>181</v>
+        <v>133</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>176</v>
+        <v>134</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>19</v>
+        <v>124</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F78" s="5" t="s">
-        <v>182</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F78" s="5"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>183</v>
+        <v>135</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>176</v>
+        <v>136</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>19</v>
+        <v>124</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F79" s="5" t="s">
-        <v>184</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F79" s="5"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>185</v>
+        <v>140</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>176</v>
+        <v>141</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>19</v>
+        <v>142</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F80" s="5" t="s">
-        <v>186</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F80" s="5"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>187</v>
+        <v>143</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>176</v>
+        <v>144</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>19</v>
+        <v>142</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F81" s="5" t="s">
-        <v>188</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F81" s="5"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>189</v>
+        <v>145</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>19</v>
+        <v>142</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F82" s="5" t="s">
-        <v>190</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F82" s="5"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>191</v>
+        <v>147</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>176</v>
+        <v>148</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>19</v>
+        <v>142</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F83" s="5" t="s">
-        <v>192</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F83" s="5"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>193</v>
+        <v>158</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>176</v>
+        <v>159</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>19</v>
+        <v>151</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F84" s="5" t="s">
-        <v>194</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F84" s="5"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>17</v>
+        <v>171</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>19</v>
+        <v>164</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F85" s="5" t="s">
-        <v>195</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F85" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:F85" xr:uid="{B3B35E5E-930D-451E-AF51-3EC3A4F9D310}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:E75">
-    <sortCondition ref="D2:D75"/>
-    <sortCondition ref="B2:B75"/>
+  <autoFilter ref="B1:F85" xr:uid="{B3B35E5E-930D-451E-AF51-3EC3A4F9D310}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:F85">
+      <sortCondition ref="E1:E85"/>
+    </sortState>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:E86">
+    <sortCondition ref="E2:E86"/>
+    <sortCondition ref="D2:D86"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>